<commit_message>
fix(redirects): use products path instead of urun
</commit_message>
<xml_diff>
--- a/dizin.xlsx
+++ b/dizin.xlsx
@@ -3047,7 +3047,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="1">
@@ -3111,7 +3111,7 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B24" s="1">
@@ -9719,7 +9719,7 @@
       </c>
     </row>
     <row r="850" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A850" t="s">
+      <c r="A850" s="2" t="s">
         <v>850</v>
       </c>
       <c r="B850" s="1">
@@ -9759,7 +9759,7 @@
       </c>
     </row>
     <row r="855" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A855" t="s">
+      <c r="A855" s="2" t="s">
         <v>855</v>
       </c>
       <c r="B855" s="1">
@@ -9769,6 +9769,10 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A45" r:id="rId1"/>
+    <hyperlink ref="A855" r:id="rId2"/>
+    <hyperlink ref="A850" r:id="rId3"/>
+    <hyperlink ref="A16" r:id="rId4"/>
+    <hyperlink ref="A24" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>